<commit_message>
Fix Streamlit Cloud rerun bug: make app.py self-contained and eliminate import recursion
</commit_message>
<xml_diff>
--- a/data/sample_clients/tata_motors_fy24/deliverables/Tata_Motors_Limited_CARO_2020_Workpaper.xlsx
+++ b/data/sample_clients/tata_motors_fy24/deliverables/Tata_Motors_Limited_CARO_2020_Workpaper.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>75.0% of OM</t>
+          <t>75% of OM</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>5.0% of OM</t>
+          <t>5% of OM</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">

</xml_diff>